<commit_message>
BWI sync — 2026-10-12 09:30 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Albania.xlsx
+++ b/BWI/bestwine_output/bestwine_Albania.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA42"/>
+  <dimension ref="A1:AA43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4732,6 +4732,71 @@
       <c r="Z42" s="2" t="inlineStr"/>
       <c r="AA42" s="2" t="inlineStr"/>
     </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Astrit Kasmi Distribution</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr"/>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>168942</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Albania</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Lezhe</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Albania</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Gjorem Km 4</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>1768</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.astritkasmi-distribution.com</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr"/>
+      <c r="M43" s="2" t="inlineStr"/>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>info@astritkasmi-distribution.com</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr"/>
+      <c r="P43" s="2" t="inlineStr"/>
+      <c r="Q43" s="2" t="inlineStr"/>
+      <c r="R43" s="2" t="inlineStr"/>
+      <c r="S43" s="2" t="inlineStr"/>
+      <c r="T43" s="2" t="inlineStr"/>
+      <c r="U43" s="2" t="inlineStr"/>
+      <c r="V43" s="2" t="inlineStr"/>
+      <c r="W43" s="2" t="inlineStr"/>
+      <c r="X43" s="2" t="inlineStr"/>
+      <c r="Y43" s="2" t="inlineStr"/>
+      <c r="Z43" s="2" t="inlineStr"/>
+      <c r="AA43" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>